<commit_message>
Sync public research package documentation and metadata
</commit_message>
<xml_diff>
--- a/data/annotations/A1.xlsx
+++ b/data/annotations/A1.xlsx
@@ -36,7 +36,7 @@
     <x:t xml:space="preserve">Source language</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Retained as supplied; no translation normalization</x:t>
+    <x:t xml:space="preserve">Source text in its supplied language</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Annotator code</x:t>
@@ -45,13 +45,13 @@
     <x:t xml:space="preserve">A1</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Date started</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">2026-08-12T03:54</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Date completed</x:t>
+    <x:t xml:space="preserve"/>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"/>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"/>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Workbook status</x:t>
@@ -147,7 +147,7 @@
     <x:t xml:space="preserve">Plan/policy disposition</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Completion Timestamp — ISO 8601 recommended (YYYY-MM-DDThh:mm).</x:t>
+    <x:t xml:space="preserve"/>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Record No</x:t>

</xml_diff>